<commit_message>
step 7: Write oil-bulletin.test.ts example tests over the excerpts
</commit_message>
<xml_diff>
--- a/src/lib/sources/__recorded__/oil-bulletin-prices-with-taxes.xlsx
+++ b/src/lib/sources/__recorded__/oil-bulletin-prices-with-taxes.xlsx
@@ -3626,6 +3626,220 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac xr xr2 xr3" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CA927381-2321-4E76-ABDE-097DEEBA8342}"><dimension ref="A1:HR1118"/><sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/><cols><col min="2" max="2" width="5.7109375" customWidth="1"/><col min="3" max="8" width="10.7109375" customWidth="1"/><col min="9" max="9" width="5.7109375" customWidth="1"/><col min="10" max="15" width="10.7109375" customWidth="1"/><col min="16" max="16" width="5.7109375" customWidth="1"/><col min="17" max="22" width="10.7109375" customWidth="1"/><col min="23" max="23" width="5.7109375" customWidth="1"/><col min="24" max="29" width="10.7109375" customWidth="1"/><col min="30" max="30" width="5.7109375" customWidth="1"/><col min="31" max="37" width="10.7109375" customWidth="1"/><col min="38" max="38" width="5.7109375" customWidth="1"/><col min="39" max="45" width="10.7109375" customWidth="1"/><col min="46" max="46" width="5.7109375" customWidth="1"/><col min="47" max="53" width="10.7109375" customWidth="1"/><col min="54" max="54" width="5.7109375" customWidth="1"/><col min="55" max="60" width="10.7109375" customWidth="1"/><col min="61" max="61" width="5.7109375" customWidth="1"/><col min="62" max="68" width="10.7109375" customWidth="1"/><col min="69" max="69" width="5.7109375" customWidth="1"/><col min="70" max="76" width="10.7109375" customWidth="1"/><col min="77" max="77" width="5.7109375" customWidth="1"/><col min="78" max="83" width="10.7109375" customWidth="1"/><col min="84" max="84" width="5.7109375" customWidth="1"/><col min="85" max="90" width="10.7109375" customWidth="1"/><col min="91" max="91" width="5.7109375" customWidth="1"/><col min="92" max="97" width="10.7109375" customWidth="1"/><col min="98" max="98" width="5.7109375" customWidth="1"/><col min="99" max="104" width="10.7109375" customWidth="1"/><col min="105" max="105" width="5.7109375" customWidth="1"/><col min="106" max="112" width="10.7109375" customWidth="1"/><col min="113" max="113" width="5.7109375" customWidth="1"/><col min="114" max="120" width="10.7109375" customWidth="1"/><col min="121" max="121" width="5.7109375" customWidth="1"/><col min="122" max="127" width="10.7109375" customWidth="1"/><col min="128" max="128" width="5.7109375" customWidth="1"/><col min="129" max="134" width="10.7109375" customWidth="1"/><col min="135" max="135" width="5.7109375" customWidth="1"/><col min="136" max="142" width="10.7109375" customWidth="1"/><col min="143" max="143" width="5.7109375" customWidth="1"/><col min="144" max="149" width="10.7109375" customWidth="1"/><col min="150" max="150" width="5.7109375" customWidth="1"/><col min="151" max="157" width="10.7109375" customWidth="1"/><col min="158" max="158" width="5.7109375" customWidth="1"/><col min="159" max="164" width="10.7109375" customWidth="1"/><col min="165" max="165" width="5.7109375" customWidth="1"/><col min="166" max="171" width="10.7109375" customWidth="1"/><col min="172" max="172" width="5.7109375" customWidth="1"/><col min="173" max="179" width="10.7109375" customWidth="1"/><col min="180" max="180" width="5.7109375" customWidth="1"/><col min="181" max="186" width="10.7109375" customWidth="1"/><col min="187" max="187" width="5.7109375" customWidth="1"/><col min="188" max="194" width="10.7109375" customWidth="1"/><col min="195" max="195" width="5.7109375" customWidth="1"/><col min="196" max="202" width="10.7109375" customWidth="1"/><col min="203" max="203" width="5.7109375" customWidth="1"/><col min="204" max="210" width="10.7109375" customWidth="1"/><col min="211" max="211" width="5.7109375" customWidth="1"/><col min="212" max="218" width="10.7109375" customWidth="1"/><col min="219" max="219" width="5.7109375" customWidth="1"/><col min="220" max="226" width="10.7109375" customWidth="1"/></cols><sheetData><row r="1" spans="1:226" x14ac:dyDescent="0.25"><c r="A1" s="27" t="s"><v>247</v></c><c r="B1" s="2" t="s"><v>1</v></c><c r="C1" s="3" t="s"><v>249</v></c><c r="D1" s="3" t="s"><v>250</v></c></row><row r="2" spans="1:226" ht="135" x14ac:dyDescent="0.25"><c r="A2" s="28"/><row r="3" spans="1:226" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"><c r="A3" s="29" t="s"><v>248</v></c><c r="B3" s="34"/><row r="4" spans="1:226" x14ac:dyDescent="0.25"><c r="A4" s="124"><v>46321</v></c><c r="B4" s="123" t="s"><v>206</v></c><c r="C4" s="110"><v>1954.0378712134029</v></c><c r="D4" s="110"><v>2146.1859738900539</v></c><row r="5" spans="1:226" x14ac:dyDescent="0.25"><c r="A5" s="43"><v>46314</v></c><c r="B5" s="123" t="s"><v>206</v></c><c r="C5" s="110"><v>1991.3323259570577</v></c><c r="D5" s="110"><v>2138.6756134933908</v></c><row r="6" spans="1:226" x14ac:dyDescent="0.25"><c r="A6" s="43"><v>46307</v></c><c r="B6" s="123" t="s"><v>206</v></c><c r="C6" s="110"><v>2009.6736867623586</v></c><c r="D6" s="110"><v>2135.7209073916079</v></c><row r="107" spans="1:226" x14ac:dyDescent="0.25"><c r="A107" s="21"><v>45600</v></c><c r="B107" s="86" t="s"><v>206</v></c><c r="C107" s="179"><v>1629.2663410422444</v></c><c r="D107" s="179"><v>1524.580178432713</v></c><row r="133" spans="1:226" x14ac:dyDescent="0.25"><c r="A133" s="21"><v>45418</v></c><c r="B133" s="86" t="s"><v>206</v></c><c r="C133" s="179"><v>1791.3149889844324</v></c><c r="D133" s="179"><v>1645.194212158339</v></c><row r="181" spans="1:226" x14ac:dyDescent="0.25"><c r="A181" s="21"><v>45082</v></c><c r="B181" s="17" t="s"><v>206</v></c><c r="C181" s="158"><v>1711.9476883475709</v></c><c r="D181" s="158"><v>1533.7807458860927</v></c><row r="182" spans="1:226" x14ac:dyDescent="0.25"><c r="A182" s="21"><v>45075</v></c><c r="B182" s="17" t="s"><v>206</v></c><c r="C182" s="158"><v>1714.7314406419894</v></c><c r="D182" s="158"><v>1534.0796445580536</v></c><row r="1096" spans="1:226" x14ac:dyDescent="0.25"><c r="A1096" t="s"><v>220</v></c></row><row r="1097" spans="1:226" x14ac:dyDescent="0.25"><c r="B1097" t="s"><v>417</v></c></row></sheetData><phoneticPr fontId="4" type="noConversion"/><pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/><pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/><legacyDrawing r:id="rId2"/></worksheet>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA927381-2321-4E76-ABDE-097DEEBA8342}">
+  <dimension ref="A1:HR1118"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="5.7109375" customWidth="1"/>
+    <col min="3" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="5.7109375" customWidth="1"/>
+    <col min="10" max="15" width="10.7109375" customWidth="1"/>
+    <col min="16" max="16" width="5.7109375" customWidth="1"/>
+    <col min="17" max="22" width="10.7109375" customWidth="1"/>
+    <col min="23" max="23" width="5.7109375" customWidth="1"/>
+    <col min="24" max="29" width="10.7109375" customWidth="1"/>
+    <col min="30" max="30" width="5.7109375" customWidth="1"/>
+    <col min="31" max="37" width="10.7109375" customWidth="1"/>
+    <col min="38" max="38" width="5.7109375" customWidth="1"/>
+    <col min="39" max="45" width="10.7109375" customWidth="1"/>
+    <col min="46" max="46" width="5.7109375" customWidth="1"/>
+    <col min="47" max="53" width="10.7109375" customWidth="1"/>
+    <col min="54" max="54" width="5.7109375" customWidth="1"/>
+    <col min="55" max="60" width="10.7109375" customWidth="1"/>
+    <col min="61" max="61" width="5.7109375" customWidth="1"/>
+    <col min="62" max="68" width="10.7109375" customWidth="1"/>
+    <col min="69" max="69" width="5.7109375" customWidth="1"/>
+    <col min="70" max="76" width="10.7109375" customWidth="1"/>
+    <col min="77" max="77" width="5.7109375" customWidth="1"/>
+    <col min="78" max="83" width="10.7109375" customWidth="1"/>
+    <col min="84" max="84" width="5.7109375" customWidth="1"/>
+    <col min="85" max="90" width="10.7109375" customWidth="1"/>
+    <col min="91" max="91" width="5.7109375" customWidth="1"/>
+    <col min="92" max="97" width="10.7109375" customWidth="1"/>
+    <col min="98" max="98" width="5.7109375" customWidth="1"/>
+    <col min="99" max="104" width="10.7109375" customWidth="1"/>
+    <col min="105" max="105" width="5.7109375" customWidth="1"/>
+    <col min="106" max="112" width="10.7109375" customWidth="1"/>
+    <col min="113" max="113" width="5.7109375" customWidth="1"/>
+    <col min="114" max="120" width="10.7109375" customWidth="1"/>
+    <col min="121" max="121" width="5.7109375" customWidth="1"/>
+    <col min="122" max="127" width="10.7109375" customWidth="1"/>
+    <col min="128" max="128" width="5.7109375" customWidth="1"/>
+    <col min="129" max="134" width="10.7109375" customWidth="1"/>
+    <col min="135" max="135" width="5.7109375" customWidth="1"/>
+    <col min="136" max="142" width="10.7109375" customWidth="1"/>
+    <col min="143" max="143" width="5.7109375" customWidth="1"/>
+    <col min="144" max="149" width="10.7109375" customWidth="1"/>
+    <col min="150" max="150" width="5.7109375" customWidth="1"/>
+    <col min="151" max="157" width="10.7109375" customWidth="1"/>
+    <col min="158" max="158" width="5.7109375" customWidth="1"/>
+    <col min="159" max="164" width="10.7109375" customWidth="1"/>
+    <col min="165" max="165" width="5.7109375" customWidth="1"/>
+    <col min="166" max="171" width="10.7109375" customWidth="1"/>
+    <col min="172" max="172" width="5.7109375" customWidth="1"/>
+    <col min="173" max="179" width="10.7109375" customWidth="1"/>
+    <col min="180" max="180" width="5.7109375" customWidth="1"/>
+    <col min="181" max="186" width="10.7109375" customWidth="1"/>
+    <col min="187" max="187" width="5.7109375" customWidth="1"/>
+    <col min="188" max="194" width="10.7109375" customWidth="1"/>
+    <col min="195" max="195" width="5.7109375" customWidth="1"/>
+    <col min="196" max="202" width="10.7109375" customWidth="1"/>
+    <col min="203" max="203" width="5.7109375" customWidth="1"/>
+    <col min="204" max="210" width="10.7109375" customWidth="1"/>
+    <col min="211" max="211" width="5.7109375" customWidth="1"/>
+    <col min="212" max="218" width="10.7109375" customWidth="1"/>
+    <col min="219" max="219" width="5.7109375" customWidth="1"/>
+    <col min="220" max="226" width="10.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
+        <v>247</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="2" spans="1:226" ht="135" x14ac:dyDescent="0.25">
+      <c r="A2" s="28"/>
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:226" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
+        <v>248</v>
+      </c>
+      <c r="B3" s="34"/>
+      <c r="C3" s="29" t="s">
+        <v>415</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="4" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A4" s="124">
+        <v>46321</v>
+      </c>
+      <c r="B4" s="123" t="s">
+        <v>206</v>
+      </c>
+      <c r="C4" s="110">
+        <v>1954.0378712134029</v>
+      </c>
+      <c r="D4" s="110">
+        <v>2146.1859738900539</v>
+      </c>
+    </row>
+    <row r="5" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A5" s="43">
+        <v>46314</v>
+      </c>
+      <c r="B5" s="123" t="s">
+        <v>206</v>
+      </c>
+      <c r="C5" s="110">
+        <v>1991.3323259570577</v>
+      </c>
+      <c r="D5" s="110">
+        <v>2138.6756134933908</v>
+      </c>
+    </row>
+    <row r="6" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A6" s="43">
+        <v>46307</v>
+      </c>
+      <c r="B6" s="123" t="s">
+        <v>206</v>
+      </c>
+      <c r="C6" s="110">
+        <v>2009.6736867623586</v>
+      </c>
+      <c r="D6" s="110">
+        <v>2135.7209073916079</v>
+      </c>
+    </row>
+    <row r="107" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A107" s="21">
+        <v>45600</v>
+      </c>
+      <c r="B107" s="86" t="s">
+        <v>206</v>
+      </c>
+      <c r="C107" s="179">
+        <v>1629.2663410422444</v>
+      </c>
+      <c r="D107" s="179">
+        <v>1524.580178432713</v>
+      </c>
+    </row>
+    <row r="133" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A133" s="21">
+        <v>45418</v>
+      </c>
+      <c r="B133" s="86" t="s">
+        <v>206</v>
+      </c>
+      <c r="C133" s="179">
+        <v>1791.3149889844324</v>
+      </c>
+      <c r="D133" s="179">
+        <v>1645.194212158339</v>
+      </c>
+    </row>
+    <row r="181" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A181" s="21">
+        <v>45082</v>
+      </c>
+      <c r="B181" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="C181" s="158">
+        <v>1711.9476883475709</v>
+      </c>
+      <c r="D181" s="158">
+        <v>1533.7807458860927</v>
+      </c>
+    </row>
+    <row r="182" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A182" s="21">
+        <v>45075</v>
+      </c>
+      <c r="B182" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="C182" s="158">
+        <v>1714.7314406419894</v>
+      </c>
+      <c r="D182" s="158">
+        <v>1534.0796445580536</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="A1096" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:226" x14ac:dyDescent="0.25">
+      <c r="B1097" t="s">
+        <v>417</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>